<commit_message>
Ordenamiento de las correcciones
</commit_message>
<xml_diff>
--- a/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES.xlsx
+++ b/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES.xlsx
@@ -1,22 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\CORRECCIONES TESIS AGOSTO 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angel\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FC2D9D4-6905-4378-B039-C0F8FEC20843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A95BC7-F7B4-432F-9B7C-3A682185E90F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-165" yWindow="-165" windowWidth="77130" windowHeight="21210" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
     <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
+    <sheet name="Hoja4" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Hoja4!$B$1:$D$22</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -27,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="81">
   <si>
     <t>Director(es) que lo solicita</t>
   </si>
@@ -399,12 +403,18 @@
   <si>
     <t>CAP 6</t>
   </si>
+  <si>
+    <t>Estatus</t>
+  </si>
+  <si>
+    <t>Cumplido</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -472,16 +482,35 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF66CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -504,11 +533,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -525,12 +569,47 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF66CC"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -805,15 +884,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="58" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -823,8 +903,11 @@
       <c r="C1" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D1" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -834,8 +917,11 @@
       <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D2" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -845,8 +931,11 @@
       <c r="C3" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D3" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -856,8 +945,9 @@
       <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -867,8 +957,9 @@
       <c r="C5" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:4" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -878,8 +969,9 @@
       <c r="C6" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -889,8 +981,9 @@
       <c r="C7" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -900,8 +993,9 @@
       <c r="C8" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
@@ -911,8 +1005,9 @@
       <c r="C9" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
@@ -922,8 +1017,9 @@
       <c r="C10" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -933,8 +1029,9 @@
       <c r="C11" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
@@ -944,8 +1041,9 @@
       <c r="C12" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
@@ -955,8 +1053,9 @@
       <c r="C13" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D13" s="2"/>
+    </row>
+    <row r="14" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
@@ -966,8 +1065,9 @@
       <c r="C14" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D14" s="2"/>
+    </row>
+    <row r="15" spans="1:4" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -977,8 +1077,9 @@
       <c r="C15" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>25</v>
       </c>
@@ -988,8 +1089,9 @@
       <c r="C16" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D16" s="2"/>
+    </row>
+    <row r="17" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>1</v>
       </c>
@@ -999,8 +1101,9 @@
       <c r="C17" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>36</v>
       </c>
@@ -1010,8 +1113,9 @@
       <c r="C18" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>4</v>
       </c>
@@ -1021,8 +1125,9 @@
       <c r="C19" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>4</v>
       </c>
@@ -1032,8 +1137,9 @@
       <c r="C20" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>41</v>
       </c>
@@ -1043,8 +1149,9 @@
       <c r="C21" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" spans="1:4" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>9</v>
       </c>
@@ -1054,8 +1161,14 @@
       <c r="C22" s="2" t="s">
         <v>45</v>
       </c>
+      <c r="D22" s="2"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A2:D22">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>$D$2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1063,12 +1176,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80CD9C86-BB81-45D2-B52F-9BBB3BE4D29C}">
   <dimension ref="B2:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="46.5703125" customWidth="1"/>
+    <col min="4" max="4" width="46.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="5" t="s">
         <v>49</v>
       </c>
@@ -1079,7 +1192,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
         <v>48</v>
       </c>
@@ -1090,7 +1203,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>48</v>
       </c>
@@ -1101,7 +1214,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>48</v>
       </c>
@@ -1112,7 +1225,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>48</v>
       </c>
@@ -1123,7 +1236,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>48</v>
       </c>
@@ -1134,7 +1247,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>48</v>
       </c>
@@ -1145,7 +1258,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>48</v>
       </c>
@@ -1165,9 +1278,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0E9ECB9-9509-4435-9143-07DA83ABD06A}">
   <dimension ref="B2:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="5" t="s">
         <v>49</v>
       </c>
@@ -1178,7 +1291,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
         <v>62</v>
       </c>
@@ -1189,7 +1302,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>62</v>
       </c>
@@ -1200,7 +1313,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>62</v>
       </c>
@@ -1211,7 +1324,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>62</v>
       </c>
@@ -1222,7 +1335,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>62</v>
       </c>
@@ -1233,7 +1346,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>62</v>
       </c>
@@ -1244,7 +1357,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>62</v>
       </c>
@@ -1255,7 +1368,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="5" t="s">
         <v>62</v>
       </c>
@@ -1266,7 +1379,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B11" s="5" t="s">
         <v>62</v>
       </c>
@@ -1277,7 +1390,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B12" s="5" t="s">
         <v>62</v>
       </c>
@@ -1288,7 +1401,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
         <v>62</v>
       </c>
@@ -1299,7 +1412,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
         <v>62</v>
       </c>
@@ -1310,7 +1423,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>62</v>
       </c>
@@ -1321,7 +1434,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>62</v>
       </c>
@@ -1335,4 +1448,264 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9318431B-ADA9-43B9-8F56-BA9994346673}">
+  <dimension ref="B1:D22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="206.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B1" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B2" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B3" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B4" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B6" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B7" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B8" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B9" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B10" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B11" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B12" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B13" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B14" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B15" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B16" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B17" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B18" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B19" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B20" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B21" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B22" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B1:D22" xr:uid="{9318431B-ADA9-43B9-8F56-BA9994346673}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:D22">
+      <sortCondition ref="C1:C22"/>
+    </sortState>
+  </autoFilter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Correcciones de primer capitulo
</commit_message>
<xml_diff>
--- a/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES.xlsx
+++ b/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angel\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A95BC7-F7B4-432F-9B7C-3A682185E90F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0FFCE48-66F4-419D-91EA-82C108B6F192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34510" yWindow="-110" windowWidth="34620" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="81">
   <si>
     <t>Director(es) que lo solicita</t>
   </si>
@@ -885,15 +885,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="58" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.44140625" customWidth="1"/>
+    <col min="3" max="3" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -907,7 +907,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -921,7 +921,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -935,7 +935,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -945,9 +945,11 @@
       <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="2"/>
-    </row>
-    <row r="5" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D4" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -957,9 +959,11 @@
       <c r="C5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="2"/>
-    </row>
-    <row r="6" spans="1:4" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D5" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -969,9 +973,11 @@
       <c r="C6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="7" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D6" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -981,9 +987,11 @@
       <c r="C7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D7" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -993,9 +1001,11 @@
       <c r="C8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D8" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
@@ -1007,7 +1017,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
@@ -1019,7 +1029,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -1031,7 +1041,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
@@ -1043,7 +1053,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
@@ -1055,7 +1065,7 @@
       </c>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
@@ -1067,7 +1077,7 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="15" spans="1:4" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -1079,7 +1089,7 @@
       </c>
       <c r="D15" s="2"/>
     </row>
-    <row r="16" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>25</v>
       </c>
@@ -1091,7 +1101,7 @@
       </c>
       <c r="D16" s="2"/>
     </row>
-    <row r="17" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>1</v>
       </c>
@@ -1103,7 +1113,7 @@
       </c>
       <c r="D17" s="2"/>
     </row>
-    <row r="18" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>36</v>
       </c>
@@ -1115,7 +1125,7 @@
       </c>
       <c r="D18" s="2"/>
     </row>
-    <row r="19" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>4</v>
       </c>
@@ -1127,7 +1137,7 @@
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>4</v>
       </c>
@@ -1139,7 +1149,7 @@
       </c>
       <c r="D20" s="2"/>
     </row>
-    <row r="21" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>41</v>
       </c>
@@ -1151,7 +1161,7 @@
       </c>
       <c r="D21" s="2"/>
     </row>
-    <row r="22" spans="1:4" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>9</v>
       </c>
@@ -1176,12 +1186,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80CD9C86-BB81-45D2-B52F-9BBB3BE4D29C}">
   <dimension ref="B2:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="46.5546875" customWidth="1"/>
+    <col min="4" max="4" width="46.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>49</v>
       </c>
@@ -1192,7 +1202,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>48</v>
       </c>
@@ -1203,7 +1213,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
         <v>48</v>
       </c>
@@ -1214,7 +1224,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
         <v>48</v>
       </c>
@@ -1225,7 +1235,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>48</v>
       </c>
@@ -1236,7 +1246,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="5" t="s">
         <v>48</v>
       </c>
@@ -1247,7 +1257,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>48</v>
       </c>
@@ -1258,7 +1268,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>48</v>
       </c>
@@ -1278,9 +1288,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0E9ECB9-9509-4435-9143-07DA83ABD06A}">
   <dimension ref="B2:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>49</v>
       </c>
@@ -1291,7 +1301,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>62</v>
       </c>
@@ -1302,7 +1312,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
         <v>62</v>
       </c>
@@ -1313,7 +1323,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
         <v>62</v>
       </c>
@@ -1324,7 +1334,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>62</v>
       </c>
@@ -1335,7 +1345,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="5" t="s">
         <v>62</v>
       </c>
@@ -1346,7 +1356,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>62</v>
       </c>
@@ -1357,7 +1367,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>62</v>
       </c>
@@ -1368,7 +1378,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="5" t="s">
         <v>62</v>
       </c>
@@ -1379,7 +1389,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B11" s="5" t="s">
         <v>62</v>
       </c>
@@ -1390,7 +1400,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B12" s="5" t="s">
         <v>62</v>
       </c>
@@ -1401,7 +1411,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B13" s="5" t="s">
         <v>62</v>
       </c>
@@ -1412,7 +1422,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="5" t="s">
         <v>62</v>
       </c>
@@ -1423,7 +1433,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
         <v>62</v>
       </c>
@@ -1434,7 +1444,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>62</v>
       </c>
@@ -1453,12 +1463,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9318431B-ADA9-43B9-8F56-BA9994346673}">
   <dimension ref="B1:D22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="206.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="206.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B1" s="11" t="s">
         <v>49</v>
       </c>
@@ -1469,7 +1479,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B2" s="12" t="s">
         <v>62</v>
       </c>
@@ -1480,7 +1490,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="12" t="s">
         <v>62</v>
       </c>
@@ -1491,7 +1501,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="12" t="s">
         <v>62</v>
       </c>
@@ -1502,7 +1512,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="12" t="s">
         <v>62</v>
       </c>
@@ -1513,7 +1523,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="12" t="s">
         <v>62</v>
       </c>
@@ -1524,7 +1534,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="12" t="s">
         <v>62</v>
       </c>
@@ -1535,7 +1545,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
         <v>48</v>
       </c>
@@ -1546,7 +1556,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
         <v>62</v>
       </c>
@@ -1557,7 +1567,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
         <v>62</v>
       </c>
@@ -1568,7 +1578,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
         <v>48</v>
       </c>
@@ -1579,7 +1589,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
         <v>48</v>
       </c>
@@ -1590,7 +1600,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
         <v>48</v>
       </c>
@@ -1601,7 +1611,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
         <v>62</v>
       </c>
@@ -1612,7 +1622,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
         <v>48</v>
       </c>
@@ -1623,7 +1633,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="8" t="s">
         <v>48</v>
       </c>
@@ -1634,7 +1644,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="8" t="s">
         <v>48</v>
       </c>
@@ -1645,7 +1655,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B18" s="12" t="s">
         <v>62</v>
       </c>
@@ -1656,7 +1666,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B19" s="12" t="s">
         <v>62</v>
       </c>
@@ -1667,7 +1677,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="20" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B20" s="12" t="s">
         <v>62</v>
       </c>
@@ -1678,7 +1688,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
         <v>62</v>
       </c>
@@ -1689,7 +1699,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B22" s="12" t="s">
         <v>62</v>
       </c>

</xml_diff>

<commit_message>
Avances hasta el marco Teorico
</commit_message>
<xml_diff>
--- a/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES.xlsx
+++ b/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0FFCE48-66F4-419D-91EA-82C108B6F192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{775CD2A7-4D02-46B2-86B5-0EEF71D1676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-34510" yWindow="-110" windowWidth="34620" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="83">
   <si>
     <t>Director(es) que lo solicita</t>
   </si>
@@ -156,16 +156,7 @@
     <t>Capítulo 2 (Marco Teórico)</t>
   </si>
   <si>
-    <t>Precisar a lo largo de los capítulos que la "no linealidad" se refiere a la separabilidad, no a los datos. Centrar el final de los capítulos en la necesidad de visualización.</t>
-  </si>
-  <si>
-    <t>Capítulos 2 y 3</t>
-  </si>
-  <si>
     <t>Dra. Adriana / Reunión</t>
-  </si>
-  <si>
-    <t>Incluir el diagrama del esquema general de un algoritmo genético (Población $\rightarrow$ Selección $\rightarrow$ Cruza $\rightarrow$ Muta, etc.).</t>
   </si>
   <si>
     <t>Capítulo 2 (Sección 2.5)</t>
@@ -408,6 +399,21 @@
   </si>
   <si>
     <t>Cumplido</t>
+  </si>
+  <si>
+    <t>Precisar a lo largo de los capítulos que la "no linealidad" se refiere a la separabilidad, no a los datos</t>
+  </si>
+  <si>
+    <t>Centrar el final de los capítulos en la necesidad de visualización.</t>
+  </si>
+  <si>
+    <t>Capitulo 2</t>
+  </si>
+  <si>
+    <t>Capitulo 3</t>
+  </si>
+  <si>
+    <t>Incluir el diagrama del esquema general de un algoritmo genético (Población -&gt; Selección -&gt; Cruza -&gt; Muta, etc.).</t>
   </si>
 </sst>
 </file>
@@ -552,7 +558,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -588,11 +594,34 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -884,7 +913,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
@@ -898,13 +927,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -918,7 +947,7 @@
         <v>3</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -932,7 +961,7 @@
         <v>6</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -946,7 +975,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -960,7 +989,7 @@
         <v>8</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -974,7 +1003,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -988,7 +1017,7 @@
         <v>13</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -1002,7 +1031,7 @@
         <v>15</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -1015,7 +1044,9 @@
       <c r="C9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="2"/>
+      <c r="D9" s="2" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="10" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
@@ -1027,53 +1058,61 @@
       <c r="C10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D10" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="B12" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="2"/>
-    </row>
-    <row r="13" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D12" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>26</v>
+        <v>1</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>79</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="14" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="D14" s="2"/>
     </row>
@@ -1082,99 +1121,133 @@
         <v>22</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="2"/>
+    </row>
+    <row r="17" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="2"/>
-    </row>
-    <row r="17" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D17" s="2"/>
-    </row>
-    <row r="18" spans="1:4" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="D18" s="2"/>
     </row>
     <row r="19" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" spans="1:4" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B21" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="2"/>
+    </row>
+    <row r="23" spans="1:4" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D19" s="2"/>
-    </row>
-    <row r="20" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20" s="2" t="s">
+      <c r="B23" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D20" s="2"/>
-    </row>
-    <row r="21" spans="1:4" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
+      <c r="D23" s="2"/>
+    </row>
+    <row r="24" spans="1:4" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D21" s="2"/>
-    </row>
-    <row r="22" spans="1:4" ht="72" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D22" s="2"/>
+      <c r="D24" s="2"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:D22">
+  <conditionalFormatting sqref="A15:D24 A2:D12">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+      <formula>$D$2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A14:D14">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>$D$2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A13 C13:D13">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>$D$2</formula>
     </cfRule>
@@ -1193,90 +1266,90 @@
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>51</v>
-      </c>
       <c r="D3" s="6" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>58</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1292,167 +1365,167 @@
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>62</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B11" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B12" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B13" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1470,244 +1543,244 @@
   <sheetData>
     <row r="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B1" s="11" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B2" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>62</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>51</v>
-      </c>
       <c r="D8" s="9" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C17" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B18" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B19" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B20" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B22" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>